<commit_message>
Bring this mapping file to this repo too for an easier access
</commit_message>
<xml_diff>
--- a/data/fabio-exiobase-v2.xlsx
+++ b/data/fabio-exiobase-v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\MyDocuments\Projects\REMASS\food time\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3963D85B-9DAB-43E0-8015-FC789891A97F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A483543-27EB-4EA4-9B83-0D620AD8E350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{3E6DCB9B-69CA-49EB-968E-D1431267C4EB}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{3E6DCB9B-69CA-49EB-968E-D1431267C4EB}"/>
   </bookViews>
   <sheets>
     <sheet name="exiobase_products" sheetId="2" r:id="rId1"/>
@@ -11408,803 +11408,803 @@
         <v>403</v>
       </c>
       <c r="E3">
-        <f>SUM(E4:E1048576)</f>
+        <f t="shared" ref="E3:AJ3" si="0">SUM(E4:E1048576)</f>
         <v>1</v>
       </c>
       <c r="F3">
-        <f>SUM(F4:F1048576)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G3">
-        <f>SUM(G4:G1048576)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="H3">
-        <f>SUM(H4:H1048576)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="I3">
-        <f>SUM(I4:I1048576)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="J3">
-        <f>SUM(J4:J1048576)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="K3">
-        <f>SUM(K4:K1048576)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="L3">
-        <f>SUM(L4:L1048576)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="M3">
-        <f>SUM(M4:M1048576)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="N3">
-        <f>SUM(N4:N1048576)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O3">
-        <f>SUM(O4:O1048576)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="P3">
-        <f>SUM(P4:P1048576)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="Q3">
-        <f>SUM(Q4:Q1048576)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="R3">
-        <f>SUM(R4:R1048576)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="S3">
-        <f>SUM(S4:S1048576)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="T3">
-        <f>SUM(T4:T1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="U3">
-        <f>SUM(U4:U1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V3">
-        <f>SUM(V4:V1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="W3">
-        <f>SUM(W4:W1048576)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="X3">
-        <f>SUM(X4:X1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Y3">
-        <f>SUM(Y4:Y1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Z3">
-        <f>SUM(Z4:Z1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AA3">
-        <f>SUM(AA4:AA1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AB3">
-        <f>SUM(AB4:AB1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AC3">
-        <f>SUM(AC4:AC1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AD3">
-        <f>SUM(AD4:AD1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AE3">
-        <f>SUM(AE4:AE1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AF3">
-        <f>SUM(AF4:AF1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AG3">
-        <f>SUM(AG4:AG1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AH3">
-        <f>SUM(AH4:AH1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AI3">
-        <f>SUM(AI4:AI1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AJ3">
-        <f>SUM(AJ4:AJ1048576)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AK3">
-        <f>SUM(AK4:AK1048576)</f>
+        <f t="shared" ref="AK3:BP3" si="1">SUM(AK4:AK1048576)</f>
         <v>0</v>
       </c>
       <c r="AL3">
-        <f>SUM(AL4:AL1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AM3">
-        <f>SUM(AM4:AM1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AN3">
-        <f>SUM(AN4:AN1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AO3">
-        <f>SUM(AO4:AO1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AP3">
-        <f>SUM(AP4:AP1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AQ3">
-        <f>SUM(AQ4:AQ1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AR3">
-        <f>SUM(AR4:AR1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AS3">
-        <f>SUM(AS4:AS1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AT3">
-        <f>SUM(AT4:AT1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AU3">
-        <f>SUM(AU4:AU1048576)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="AV3">
-        <f>SUM(AV4:AV1048576)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="AW3">
-        <f>SUM(AW4:AW1048576)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="AX3">
-        <f>SUM(AX4:AX1048576)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="AY3">
-        <f>SUM(AY4:AY1048576)</f>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="AZ3">
-        <f>SUM(AZ4:AZ1048576)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="BA3">
-        <f>SUM(BA4:BA1048576)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="BB3">
-        <f>SUM(BB4:BB1048576)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="BC3">
-        <f>SUM(BC4:BC1048576)</f>
-        <v>41</v>
+        <f t="shared" si="1"/>
+        <v>42</v>
       </c>
       <c r="BD3">
-        <f>SUM(BD4:BD1048576)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="BE3">
-        <f>SUM(BE4:BE1048576)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="BF3">
-        <f>SUM(BF4:BF1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BG3">
-        <f>SUM(BG4:BG1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BH3">
-        <f>SUM(BH4:BH1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BI3">
-        <f>SUM(BI4:BI1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BJ3">
-        <f>SUM(BJ4:BJ1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BK3">
-        <f>SUM(BK4:BK1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BL3">
-        <f>SUM(BL4:BL1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BM3">
-        <f>SUM(BM4:BM1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BN3">
-        <f>SUM(BN4:BN1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BO3">
-        <f>SUM(BO4:BO1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BP3">
-        <f>SUM(BP4:BP1048576)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="BQ3">
-        <f>SUM(BQ4:BQ1048576)</f>
+        <f t="shared" ref="BQ3:CV3" si="2">SUM(BQ4:BQ1048576)</f>
         <v>0</v>
       </c>
       <c r="BR3">
-        <f>SUM(BR4:BR1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="BS3">
-        <f>SUM(BS4:BS1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="BT3">
-        <f>SUM(BT4:BT1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="BU3">
-        <f>SUM(BU4:BU1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="BV3">
-        <f>SUM(BV4:BV1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="BW3">
-        <f>SUM(BW4:BW1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="BX3">
-        <f>SUM(BX4:BX1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="BY3">
-        <f>SUM(BY4:BY1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="BZ3">
-        <f>SUM(BZ4:BZ1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CA3">
-        <f>SUM(CA4:CA1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CB3">
-        <f>SUM(CB4:CB1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CC3">
-        <f>SUM(CC4:CC1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CD3">
-        <f>SUM(CD4:CD1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CE3">
-        <f>SUM(CE4:CE1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CF3">
-        <f>SUM(CF4:CF1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CG3">
-        <f>SUM(CG4:CG1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CH3">
-        <f>SUM(CH4:CH1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CI3">
-        <f>SUM(CI4:CI1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CJ3">
-        <f>SUM(CJ4:CJ1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CK3">
-        <f>SUM(CK4:CK1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CL3">
-        <f>SUM(CL4:CL1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CM3">
-        <f>SUM(CM4:CM1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CN3">
-        <f>SUM(CN4:CN1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CO3">
-        <f>SUM(CO4:CO1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CP3">
-        <f>SUM(CP4:CP1048576)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="CQ3">
-        <f>SUM(CQ4:CQ1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CR3">
-        <f>SUM(CR4:CR1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CS3">
-        <f>SUM(CS4:CS1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CT3">
-        <f>SUM(CT4:CT1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CU3">
-        <f>SUM(CU4:CU1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CV3">
-        <f>SUM(CV4:CV1048576)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="CW3">
-        <f>SUM(CW4:CW1048576)</f>
+        <f t="shared" ref="CW3:EB3" si="3">SUM(CW4:CW1048576)</f>
         <v>0</v>
       </c>
       <c r="CX3">
-        <f>SUM(CX4:CX1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="CY3">
-        <f>SUM(CY4:CY1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="CZ3">
-        <f>SUM(CZ4:CZ1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DA3">
-        <f>SUM(DA4:DA1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DB3">
-        <f>SUM(DB4:DB1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DC3">
-        <f>SUM(DC4:DC1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DD3">
-        <f>SUM(DD4:DD1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DE3">
-        <f>SUM(DE4:DE1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DF3">
-        <f>SUM(DF4:DF1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DG3">
-        <f>SUM(DG4:DG1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DH3">
-        <f>SUM(DH4:DH1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DI3">
-        <f>SUM(DI4:DI1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DJ3">
-        <f>SUM(DJ4:DJ1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DK3">
-        <f>SUM(DK4:DK1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DL3">
-        <f>SUM(DL4:DL1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DM3">
-        <f>SUM(DM4:DM1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DN3">
-        <f>SUM(DN4:DN1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DO3">
-        <f>SUM(DO4:DO1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DP3">
-        <f>SUM(DP4:DP1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DQ3">
-        <f>SUM(DQ4:DQ1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DR3">
-        <f>SUM(DR4:DR1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DS3">
-        <f>SUM(DS4:DS1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DT3">
-        <f>SUM(DT4:DT1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DU3">
-        <f>SUM(DU4:DU1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DV3">
-        <f>SUM(DV4:DV1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DW3">
-        <f>SUM(DW4:DW1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DX3">
-        <f>SUM(DX4:DX1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DY3">
-        <f>SUM(DY4:DY1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="DZ3">
-        <f>SUM(DZ4:DZ1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="EA3">
-        <f>SUM(EA4:EA1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="EB3">
-        <f>SUM(EB4:EB1048576)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="EC3">
-        <f>SUM(EC4:EC1048576)</f>
+        <f t="shared" ref="EC3:FH3" si="4">SUM(EC4:EC1048576)</f>
         <v>0</v>
       </c>
       <c r="ED3">
-        <f>SUM(ED4:ED1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EE3">
-        <f>SUM(EE4:EE1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EF3">
-        <f>SUM(EF4:EF1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EG3">
-        <f>SUM(EG4:EG1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EH3">
-        <f>SUM(EH4:EH1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EI3">
-        <f>SUM(EI4:EI1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EJ3">
-        <f>SUM(EJ4:EJ1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EK3">
-        <f>SUM(EK4:EK1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EL3">
-        <f>SUM(EL4:EL1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EM3">
-        <f>SUM(EM4:EM1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EN3">
-        <f>SUM(EN4:EN1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EO3">
-        <f>SUM(EO4:EO1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EP3">
-        <f>SUM(EP4:EP1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EQ3">
-        <f>SUM(EQ4:EQ1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="ER3">
-        <f>SUM(ER4:ER1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="ES3">
-        <f>SUM(ES4:ES1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="ET3">
-        <f>SUM(ET4:ET1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EU3">
-        <f>SUM(EU4:EU1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EV3">
-        <f>SUM(EV4:EV1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EW3">
-        <f>SUM(EW4:EW1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EX3">
-        <f>SUM(EX4:EX1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EY3">
-        <f>SUM(EY4:EY1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="EZ3">
-        <f>SUM(EZ4:EZ1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FA3">
-        <f>SUM(FA4:FA1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FB3">
-        <f>SUM(FB4:FB1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FC3">
-        <f>SUM(FC4:FC1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FD3">
-        <f>SUM(FD4:FD1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FE3">
-        <f>SUM(FE4:FE1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FF3">
-        <f>SUM(FF4:FF1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FG3">
-        <f>SUM(FG4:FG1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FH3">
-        <f>SUM(FH4:FH1048576)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="FI3">
-        <f>SUM(FI4:FI1048576)</f>
+        <f t="shared" ref="FI3:GN3" si="5">SUM(FI4:FI1048576)</f>
         <v>0</v>
       </c>
       <c r="FJ3">
-        <f>SUM(FJ4:FJ1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FK3">
-        <f>SUM(FK4:FK1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FL3">
-        <f>SUM(FL4:FL1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FM3">
-        <f>SUM(FM4:FM1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FN3">
-        <f>SUM(FN4:FN1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FO3">
-        <f>SUM(FO4:FO1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FP3">
-        <f>SUM(FP4:FP1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FQ3">
-        <f>SUM(FQ4:FQ1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FR3">
-        <f>SUM(FR4:FR1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FS3">
-        <f>SUM(FS4:FS1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FT3">
-        <f>SUM(FT4:FT1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FU3">
-        <f>SUM(FU4:FU1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FV3">
-        <f>SUM(FV4:FV1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FW3">
-        <f>SUM(FW4:FW1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FX3">
-        <f>SUM(FX4:FX1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FY3">
-        <f>SUM(FY4:FY1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="FZ3">
-        <f>SUM(FZ4:FZ1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GA3">
-        <f>SUM(GA4:GA1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GB3">
-        <f>SUM(GB4:GB1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GC3">
-        <f>SUM(GC4:GC1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GD3">
-        <f>SUM(GD4:GD1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GE3">
-        <f>SUM(GE4:GE1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GF3">
-        <f>SUM(GF4:GF1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GG3">
-        <f>SUM(GG4:GG1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GH3">
-        <f>SUM(GH4:GH1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GI3">
-        <f>SUM(GI4:GI1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GJ3">
-        <f>SUM(GJ4:GJ1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GK3">
-        <f>SUM(GK4:GK1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GL3">
-        <f>SUM(GL4:GL1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GM3">
-        <f>SUM(GM4:GM1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GN3">
-        <f>SUM(GN4:GN1048576)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="GO3">
-        <f>SUM(GO4:GO1048576)</f>
+        <f t="shared" ref="GO3:HT3" si="6">SUM(GO4:GO1048576)</f>
         <v>0</v>
       </c>
       <c r="GP3">
-        <f>SUM(GP4:GP1048576)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="GQ3">
-        <f>SUM(GQ4:GQ1048576)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="GR3">
-        <f>SUM(GR4:GR1048576)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="GS3">
-        <f>SUM(GS4:GS1048576)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="GT3">
-        <f>SUM(GT4:GT1048576)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="GU3">
-        <f>SUM(GU4:GU1048576)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="GV3">
-        <f>SUM(GV4:GV1048576)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -12219,7 +12219,7 @@
         <v>406</v>
       </c>
       <c r="D4">
-        <f t="shared" ref="D4:D67" si="0">SUM(E4:GV4)</f>
+        <f t="shared" ref="D4:D67" si="7">SUM(E4:GV4)</f>
         <v>2</v>
       </c>
       <c r="E4">
@@ -12240,7 +12240,7 @@
         <v>406</v>
       </c>
       <c r="D5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="F5">
@@ -12261,7 +12261,7 @@
         <v>406</v>
       </c>
       <c r="D6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="G6">
@@ -12282,7 +12282,7 @@
         <v>406</v>
       </c>
       <c r="D7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="G7">
@@ -12303,7 +12303,7 @@
         <v>406</v>
       </c>
       <c r="D8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="G8">
@@ -12324,7 +12324,7 @@
         <v>406</v>
       </c>
       <c r="D9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="G9">
@@ -12345,7 +12345,7 @@
         <v>406</v>
       </c>
       <c r="D10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="G10">
@@ -12366,7 +12366,7 @@
         <v>406</v>
       </c>
       <c r="D11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="G11">
@@ -12387,7 +12387,7 @@
         <v>406</v>
       </c>
       <c r="D12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="G12">
@@ -12408,7 +12408,7 @@
         <v>425</v>
       </c>
       <c r="D13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H13">
@@ -12429,7 +12429,7 @@
         <v>425</v>
       </c>
       <c r="D14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H14">
@@ -12450,7 +12450,7 @@
         <v>425</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H15">
@@ -12471,7 +12471,7 @@
         <v>425</v>
       </c>
       <c r="D16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H16">
@@ -12492,7 +12492,7 @@
         <v>425</v>
       </c>
       <c r="D17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H17">
@@ -12513,7 +12513,7 @@
         <v>436</v>
       </c>
       <c r="D18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="J18">
@@ -12531,7 +12531,7 @@
         <v>436</v>
       </c>
       <c r="D19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="J19">
@@ -12549,7 +12549,7 @@
         <v>441</v>
       </c>
       <c r="D20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H20">
@@ -12570,7 +12570,7 @@
         <v>441</v>
       </c>
       <c r="D21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H21">
@@ -12591,7 +12591,7 @@
         <v>441</v>
       </c>
       <c r="D22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H22">
@@ -12612,7 +12612,7 @@
         <v>441</v>
       </c>
       <c r="D23">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H23">
@@ -12633,7 +12633,7 @@
         <v>450</v>
       </c>
       <c r="D24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I24">
@@ -12651,7 +12651,7 @@
         <v>450</v>
       </c>
       <c r="D25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I25">
@@ -12669,7 +12669,7 @@
         <v>450</v>
       </c>
       <c r="D26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I26">
@@ -12687,7 +12687,7 @@
         <v>450</v>
       </c>
       <c r="D27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I27">
@@ -12705,7 +12705,7 @@
         <v>450</v>
       </c>
       <c r="D28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I28">
@@ -12723,7 +12723,7 @@
         <v>450</v>
       </c>
       <c r="D29">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I29">
@@ -12741,7 +12741,7 @@
         <v>450</v>
       </c>
       <c r="D30">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I30">
@@ -12759,7 +12759,7 @@
         <v>450</v>
       </c>
       <c r="D31">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I31">
@@ -12777,7 +12777,7 @@
         <v>450</v>
       </c>
       <c r="D32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I32">
@@ -12795,7 +12795,7 @@
         <v>450</v>
       </c>
       <c r="D33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I33">
@@ -12813,7 +12813,7 @@
         <v>441</v>
       </c>
       <c r="D34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H34">
@@ -12834,7 +12834,7 @@
         <v>441</v>
       </c>
       <c r="D35">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H35">
@@ -12855,7 +12855,7 @@
         <v>441</v>
       </c>
       <c r="D36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H36">
@@ -12876,7 +12876,7 @@
         <v>441</v>
       </c>
       <c r="D37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H37">
@@ -12897,7 +12897,7 @@
         <v>441</v>
       </c>
       <c r="D38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H38">
@@ -12918,7 +12918,7 @@
         <v>441</v>
       </c>
       <c r="D39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H39">
@@ -12939,7 +12939,7 @@
         <v>441</v>
       </c>
       <c r="D40">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H40">
@@ -12960,7 +12960,7 @@
         <v>441</v>
       </c>
       <c r="D41">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H41">
@@ -12981,7 +12981,7 @@
         <v>441</v>
       </c>
       <c r="D42">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H42">
@@ -13002,7 +13002,7 @@
         <v>441</v>
       </c>
       <c r="D43">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H43">
@@ -13023,7 +13023,7 @@
         <v>441</v>
       </c>
       <c r="D44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H44">
@@ -13044,7 +13044,7 @@
         <v>441</v>
       </c>
       <c r="D45">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H45">
@@ -13065,7 +13065,7 @@
         <v>441</v>
       </c>
       <c r="D46">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H46">
@@ -13086,7 +13086,7 @@
         <v>441</v>
       </c>
       <c r="D47">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="H47">
@@ -13107,7 +13107,7 @@
         <v>499</v>
       </c>
       <c r="D48">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="L48">
@@ -13128,7 +13128,7 @@
         <v>499</v>
       </c>
       <c r="D49">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="L49">
@@ -13149,7 +13149,7 @@
         <v>499</v>
       </c>
       <c r="D50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="L50">
@@ -13170,7 +13170,7 @@
         <v>441</v>
       </c>
       <c r="D51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="L51">
@@ -13188,7 +13188,7 @@
         <v>441</v>
       </c>
       <c r="D52">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="L52">
@@ -13209,7 +13209,7 @@
         <v>441</v>
       </c>
       <c r="D53">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="L53">
@@ -13230,7 +13230,7 @@
         <v>441</v>
       </c>
       <c r="D54">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="L54">
@@ -13251,7 +13251,7 @@
         <v>441</v>
       </c>
       <c r="D55">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="L55">
@@ -13272,7 +13272,7 @@
         <v>516</v>
       </c>
       <c r="D56">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K56">
@@ -13290,7 +13290,7 @@
         <v>516</v>
       </c>
       <c r="D57">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K57">
@@ -13308,7 +13308,7 @@
         <v>516</v>
       </c>
       <c r="D58">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K58">
@@ -13326,7 +13326,7 @@
         <v>516</v>
       </c>
       <c r="D59">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K59">
@@ -13344,7 +13344,7 @@
         <v>516</v>
       </c>
       <c r="D60">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K60">
@@ -13362,7 +13362,7 @@
         <v>516</v>
       </c>
       <c r="D61">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K61">
@@ -13380,7 +13380,7 @@
         <v>529</v>
       </c>
       <c r="D62">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="L62">
@@ -13398,7 +13398,7 @@
         <v>529</v>
       </c>
       <c r="D63">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="L63">
@@ -13416,7 +13416,7 @@
         <v>534</v>
       </c>
       <c r="D64">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -13431,7 +13431,7 @@
         <v>534</v>
       </c>
       <c r="D65">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -13446,7 +13446,7 @@
         <v>450</v>
       </c>
       <c r="D66">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I66">
@@ -13464,7 +13464,7 @@
         <v>450</v>
       </c>
       <c r="D67">
-        <f t="shared" si="0"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I67">
@@ -13482,7 +13482,7 @@
         <v>543</v>
       </c>
       <c r="D68">
-        <f t="shared" ref="D68:D126" si="1">SUM(E68:GV68)</f>
+        <f t="shared" ref="D68:D126" si="8">SUM(E68:GV68)</f>
         <v>1</v>
       </c>
       <c r="BB68">
@@ -13500,7 +13500,7 @@
         <v>543</v>
       </c>
       <c r="D69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="BB69">
@@ -13518,7 +13518,7 @@
         <v>543</v>
       </c>
       <c r="D70">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>2</v>
       </c>
       <c r="BC70">
@@ -13539,7 +13539,7 @@
         <v>551</v>
       </c>
       <c r="D71">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY71">
@@ -13557,7 +13557,7 @@
         <v>551</v>
       </c>
       <c r="D72">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY72">
@@ -13575,7 +13575,7 @@
         <v>551</v>
       </c>
       <c r="D73">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY73">
@@ -13593,7 +13593,7 @@
         <v>551</v>
       </c>
       <c r="D74">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY74">
@@ -13611,7 +13611,7 @@
         <v>551</v>
       </c>
       <c r="D75">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY75">
@@ -13629,7 +13629,7 @@
         <v>551</v>
       </c>
       <c r="D76">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY76">
@@ -13647,7 +13647,7 @@
         <v>551</v>
       </c>
       <c r="D77">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY77">
@@ -13665,7 +13665,7 @@
         <v>551</v>
       </c>
       <c r="D78">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY78">
@@ -13683,7 +13683,7 @@
         <v>551</v>
       </c>
       <c r="D79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY79">
@@ -13701,7 +13701,7 @@
         <v>551</v>
       </c>
       <c r="D80">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY80">
@@ -13719,7 +13719,7 @@
         <v>551</v>
       </c>
       <c r="D81">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY81">
@@ -13737,7 +13737,7 @@
         <v>551</v>
       </c>
       <c r="D82">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY82">
@@ -13755,7 +13755,7 @@
         <v>551</v>
       </c>
       <c r="D83">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY83">
@@ -13773,7 +13773,7 @@
         <v>578</v>
       </c>
       <c r="D84">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY84">
@@ -13791,7 +13791,7 @@
         <v>578</v>
       </c>
       <c r="D85">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY85">
@@ -13809,7 +13809,7 @@
         <v>578</v>
       </c>
       <c r="D86">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY86">
@@ -13827,7 +13827,7 @@
         <v>578</v>
       </c>
       <c r="D87">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY87">
@@ -13845,7 +13845,7 @@
         <v>578</v>
       </c>
       <c r="D88">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY88">
@@ -13863,7 +13863,7 @@
         <v>578</v>
       </c>
       <c r="D89">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY89">
@@ -13881,7 +13881,7 @@
         <v>578</v>
       </c>
       <c r="D90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY90">
@@ -13899,7 +13899,7 @@
         <v>578</v>
       </c>
       <c r="D91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY91">
@@ -13917,7 +13917,7 @@
         <v>578</v>
       </c>
       <c r="D92">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AY92">
@@ -13935,7 +13935,7 @@
         <v>597</v>
       </c>
       <c r="D93">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="BD93">
@@ -13953,7 +13953,7 @@
         <v>597</v>
       </c>
       <c r="D94">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="BD94">
@@ -13971,7 +13971,7 @@
         <v>597</v>
       </c>
       <c r="D95">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="BD95">
@@ -13989,7 +13989,7 @@
         <v>597</v>
       </c>
       <c r="D96">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="BD96">
@@ -14007,7 +14007,7 @@
         <v>606</v>
       </c>
       <c r="D97">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="CP97">
@@ -14025,7 +14025,7 @@
         <v>516</v>
       </c>
       <c r="D98">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="K98">
@@ -14043,7 +14043,7 @@
         <v>610</v>
       </c>
       <c r="D99">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="M99">
@@ -14061,7 +14061,7 @@
         <v>610</v>
       </c>
       <c r="D100">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P100">
@@ -14079,7 +14079,7 @@
         <v>610</v>
       </c>
       <c r="D101">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P101">
@@ -14097,7 +14097,7 @@
         <v>610</v>
       </c>
       <c r="D102">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P102">
@@ -14115,7 +14115,7 @@
         <v>610</v>
       </c>
       <c r="D103">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="N103">
@@ -14133,7 +14133,7 @@
         <v>610</v>
       </c>
       <c r="D104">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="O104">
@@ -14151,7 +14151,7 @@
         <v>610</v>
       </c>
       <c r="D105">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P105">
@@ -14169,7 +14169,7 @@
         <v>610</v>
       </c>
       <c r="D106">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P106">
@@ -14187,7 +14187,7 @@
         <v>610</v>
       </c>
       <c r="D107">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P107">
@@ -14205,7 +14205,7 @@
         <v>610</v>
       </c>
       <c r="D108">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P108">
@@ -14223,7 +14223,7 @@
         <v>610</v>
       </c>
       <c r="D109">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P109">
@@ -14241,7 +14241,7 @@
         <v>610</v>
       </c>
       <c r="D110">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P110">
@@ -14259,7 +14259,7 @@
         <v>610</v>
       </c>
       <c r="D111">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P111">
@@ -14277,7 +14277,7 @@
         <v>636</v>
       </c>
       <c r="D112">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>2</v>
       </c>
       <c r="R112">
@@ -14298,7 +14298,7 @@
         <v>636</v>
       </c>
       <c r="D113">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AZ113">
@@ -14316,7 +14316,7 @@
         <v>640</v>
       </c>
       <c r="D114">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>2</v>
       </c>
       <c r="Q114">
@@ -14337,7 +14337,7 @@
         <v>643</v>
       </c>
       <c r="D115">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="S115">
@@ -14355,7 +14355,7 @@
         <v>646</v>
       </c>
       <c r="D116">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AU116">
@@ -14373,7 +14373,7 @@
         <v>646</v>
       </c>
       <c r="D117">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AX117">
@@ -14391,7 +14391,7 @@
         <v>646</v>
       </c>
       <c r="D118">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AV118">
@@ -14409,7 +14409,7 @@
         <v>646</v>
       </c>
       <c r="D119">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AW119">
@@ -14427,7 +14427,7 @@
         <v>646</v>
       </c>
       <c r="D120">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AX120">
@@ -14445,7 +14445,7 @@
         <v>646</v>
       </c>
       <c r="D121">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AX121">
@@ -14463,7 +14463,7 @@
         <v>659</v>
       </c>
       <c r="D122">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AX122">
@@ -14481,7 +14481,7 @@
         <v>643</v>
       </c>
       <c r="D123">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AX123">
@@ -14499,7 +14499,7 @@
         <v>664</v>
       </c>
       <c r="D124">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>2</v>
       </c>
       <c r="Q124">
@@ -14520,7 +14520,7 @@
         <v>643</v>
       </c>
       <c r="D125">
-        <f t="shared" si="1"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="S125">
@@ -14538,10 +14538,13 @@
         <v>667</v>
       </c>
       <c r="D126">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f t="shared" si="8"/>
+        <v>3</v>
       </c>
       <c r="W126">
+        <v>1</v>
+      </c>
+      <c r="BC126">
         <v>1</v>
       </c>
       <c r="BE126">

</xml_diff>

<commit_message>
Remove 'processed food' (EXIO) mapping to fish product (FABIO)
</commit_message>
<xml_diff>
--- a/data/fabio-exiobase-v2.xlsx
+++ b/data/fabio-exiobase-v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\MyDocuments\Projects\REMASS\food time\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A483543-27EB-4EA4-9B83-0D620AD8E350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EB6958-B4B3-4815-BF01-5978CFBDF3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{3E6DCB9B-69CA-49EB-968E-D1431267C4EB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3E6DCB9B-69CA-49EB-968E-D1431267C4EB}"/>
   </bookViews>
   <sheets>
     <sheet name="exiobase_products" sheetId="2" r:id="rId1"/>
@@ -11609,7 +11609,7 @@
       </c>
       <c r="BC3">
         <f t="shared" si="1"/>
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="BD3">
         <f t="shared" si="1"/>
@@ -12176,7 +12176,7 @@
         <v>0</v>
       </c>
       <c r="GO3">
-        <f t="shared" ref="GO3:HT3" si="6">SUM(GO4:GO1048576)</f>
+        <f t="shared" ref="GO3:GV3" si="6">SUM(GO4:GO1048576)</f>
         <v>0</v>
       </c>
       <c r="GP3">
@@ -14539,12 +14539,9 @@
       </c>
       <c r="D126">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W126">
-        <v>1</v>
-      </c>
-      <c r="BC126">
         <v>1</v>
       </c>
       <c r="BE126">

</xml_diff>